<commit_message>
Modified reports and AI prompt
</commit_message>
<xml_diff>
--- a/static/GENEFOOD_variants_list.xlsx
+++ b/static/GENEFOOD_variants_list.xlsx
@@ -5,25 +5,25 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="12"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="11"/>
   </bookViews>
   <sheets>
-    <sheet name="BASE" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="COMPLETA" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="RIS AUMENTO DI PESO" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="RIS T2D" sheetId="4" state="visible" r:id="rId5"/>
-    <sheet name="RISC PATOLOGIE CARDIOVASCOLARI" sheetId="5" state="visible" r:id="rId6"/>
-    <sheet name="RIS PLUS" sheetId="6" state="visible" r:id="rId7"/>
-    <sheet name="RIS VITA" sheetId="7" state="visible" r:id="rId8"/>
-    <sheet name="RIS SPORT" sheetId="8" state="visible" r:id="rId9"/>
-    <sheet name="RIS AGEING" sheetId="9" state="visible" r:id="rId10"/>
-    <sheet name="RIS JUNIOR_INTOLL" sheetId="10" state="visible" r:id="rId11"/>
-    <sheet name="RIS JUNIOR_MET" sheetId="11" state="visible" r:id="rId12"/>
-    <sheet name="RIS JUNIOR_CARIE" sheetId="12" state="visible" r:id="rId13"/>
-    <sheet name="RIS JUNIOR_FRAG" sheetId="13" state="visible" r:id="rId14"/>
-    <sheet name="RIS MAMMA" sheetId="14" state="visible" r:id="rId15"/>
-    <sheet name="AGING" sheetId="15" state="visible" r:id="rId16"/>
-    <sheet name="MAMMA" sheetId="16" state="visible" r:id="rId17"/>
+    <sheet name="BASE" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="COMPLETA" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="RIS AUMENTO DI PESO" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="RIS T2D" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="RISC PATOLOGIE CARDIOVASCOLARI" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="RIS PLUS" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="RIS VITA" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="RIS SPORT" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="RIS AGEING" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="RIS JUNIOR_INTOLL" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="RIS JUNIOR_MET" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="RIS JUNIOR_CARIE" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="RIS JUNIOR_FRAG" sheetId="13" state="visible" r:id="rId15"/>
+    <sheet name="RIS MAMMA" sheetId="14" state="visible" r:id="rId16"/>
+    <sheet name="AGING" sheetId="15" state="visible" r:id="rId17"/>
+    <sheet name="MAMMA" sheetId="16" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">COMPLETA!$A$1:$H$91</definedName>
@@ -1217,7 +1217,7 @@
     <t xml:space="preserve">AC</t>
   </si>
   <si>
-    <t xml:space="preserve">HLADQA1-B1</t>
+    <t xml:space="preserve">HLA_DQA1-B1</t>
   </si>
   <si>
     <t xml:space="preserve">xxx1</t>
@@ -3100,15 +3100,15 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFFFFF"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF232629"/>
-          <bgColor rgb="FFFFFFFF"/>
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3116,6 +3116,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3123,6 +3124,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF212121"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3130,6 +3132,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF212529"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3137,6 +3140,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF333333"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3144,6 +3148,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF0070C0"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3151,6 +3156,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF33CC33"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3158,6 +3164,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3172,6 +3179,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF4B183"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3179,6 +3187,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF808080"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3186,6 +3195,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFA9D18E"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3193,6 +3203,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3228,6 +3239,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF00B050"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3244,6 +3256,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFCFCFC"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3349,8 +3362,114 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -3360,8 +3479,8 @@
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="1" width="16.29"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="2" min="2" style="1" width="3.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="21.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="21.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="16.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="30.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="27.71"/>
@@ -4390,7 +4509,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -4749,7 +4868,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="125" t="s">
         <v>488</v>
       </c>
@@ -4767,7 +4886,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="125" t="s">
         <v>488</v>
       </c>
@@ -4785,7 +4904,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="125" t="s">
         <v>488</v>
       </c>
@@ -4803,7 +4922,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="125" t="s">
         <v>488</v>
       </c>
@@ -4821,7 +4940,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="125" t="s">
         <v>488</v>
       </c>
@@ -4839,7 +4958,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="125" t="s">
         <v>488</v>
       </c>
@@ -4857,7 +4976,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="125" t="s">
         <v>488</v>
       </c>
@@ -4875,7 +4994,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="125" t="s">
         <v>488</v>
       </c>
@@ -4893,7 +5012,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="125" t="s">
         <v>488</v>
       </c>
@@ -5022,14 +5141,14 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normale"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normale"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -5874,7 +5993,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
         <v>101</v>
       </c>
@@ -5892,7 +6011,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
         <v>101</v>
       </c>
@@ -5910,7 +6029,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
         <v>101</v>
       </c>
@@ -6911,14 +7030,14 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normale"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normale"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -7582,14 +7701,14 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normale"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normale"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -8725,22 +8844,22 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normale"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normale"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G61"/>
-  <sheetFormatPr defaultColWidth="20.1640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="20.16796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="35.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="23.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="23.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="4" width="14.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="82" width="14.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="93" width="24"/>
@@ -9757,7 +9876,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -9905,7 +10024,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="107.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
         <v>158</v>
       </c>
@@ -9983,7 +10102,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="54.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
         <v>161</v>
       </c>
@@ -10009,7 +10128,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="54.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
         <v>163</v>
       </c>
@@ -10035,7 +10154,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="67.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="1" t="s">
         <v>165</v>
       </c>
@@ -10239,12 +10358,12 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L30"/>
-  <sheetFormatPr defaultColWidth="20.1640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="20.16796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="7.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="14.15"/>
@@ -11091,7 +11210,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -11104,11 +11223,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="25" width="14.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="25" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="25" width="28.14"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="8" style="27" width="9.13"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="8" style="27" width="9.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="25" width="20.71"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="11" min="10" style="25" width="9.13"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="11" min="10" style="25" width="9.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="25" width="34.13"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="13" style="25" width="9.13"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="13" style="25" width="9.12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13520,17 +13639,17 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.3046875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="27.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="21.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="3" width="18.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="17.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="17.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="41.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="20.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="3" width="14.69"/>
@@ -14030,7 +14149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
         <v>101</v>
       </c>
@@ -14044,7 +14163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
         <v>101</v>
       </c>
@@ -14058,7 +14177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
         <v>101</v>
       </c>
@@ -14118,7 +14237,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -14679,14 +14798,14 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H65"/>
-  <sheetFormatPr defaultColWidth="14.30078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.3046875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="11" width="26.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="11" width="26.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="11" width="24.29"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="3" style="11" width="14.28"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="5" style="72" width="14.28"/>
@@ -15635,7 +15754,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -15955,7 +16074,7 @@
       <c r="G16" s="85"/>
       <c r="H16" s="85"/>
     </row>
-    <row r="17" customFormat="false" ht="16.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="82" t="s">
         <v>238</v>
       </c>
@@ -15974,7 +16093,7 @@
       <c r="G17" s="85"/>
       <c r="H17" s="85"/>
     </row>
-    <row r="18" customFormat="false" ht="16.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="82" t="s">
         <v>238</v>
       </c>
@@ -15993,7 +16112,7 @@
       <c r="G18" s="86"/>
       <c r="H18" s="86"/>
     </row>
-    <row r="19" customFormat="false" ht="16.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="82" t="s">
         <v>238</v>
       </c>
@@ -16012,7 +16131,7 @@
       <c r="G19" s="86"/>
       <c r="H19" s="86"/>
     </row>
-    <row r="20" customFormat="false" ht="16.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="82" t="s">
         <v>235</v>
       </c>
@@ -16031,7 +16150,7 @@
       <c r="G20" s="87"/>
       <c r="H20" s="87"/>
     </row>
-    <row r="21" customFormat="false" ht="16.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="82" t="s">
         <v>235</v>
       </c>
@@ -16050,7 +16169,7 @@
       <c r="G21" s="87"/>
       <c r="H21" s="87"/>
     </row>
-    <row r="22" customFormat="false" ht="16.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="82" t="s">
         <v>235</v>
       </c>
@@ -16165,7 +16284,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -16178,12 +16297,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="24.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="12.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="4" width="50.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="4" width="50.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="54" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="3" width="32.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="3" width="11.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="3" width="10.59"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="12" style="3" width="9.13"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="12" style="3" width="9.12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16922,7 +17041,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -18264,7 +18383,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -18275,7 +18394,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="11" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="11" width="14.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="95" width="9.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="95" width="9.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="59.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="58.41"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1022" min="8" style="1" width="22.57"/>

</xml_diff>

<commit_message>
Some minor corrections on snp naming or coloring; Aging is now handled by the newer claude model because the report often gets too long with the 06-24 one
</commit_message>
<xml_diff>
--- a/static/GENEFOOD_variants_list.xlsx
+++ b/static/GENEFOOD_variants_list.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="11"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="BASE" sheetId="1" state="visible" r:id="rId3"/>
@@ -16161,7 +16161,7 @@
         <v>388</v>
       </c>
       <c r="E21" s="82" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="F21" s="82" t="s">
         <v>387</v>

</xml_diff>